<commit_message>
feat(closing): say what is missing — statement period, resident tax form, engine f6c10f1/9206d62
- summary chip and cash KPI say "statement ends on <date>, month end not checked" when the bank file stops early
  (before, the chip said bank and books agree — true only up to the last row)
- in-page form for "no resident tax data": special collection (amount + first month, through next May) or none
- select fields carry a title (accessibility; the test harness finds fields by title)
- engine: register vs book for fixed assets, credit balances on assets, statement period item, resident tax
  without default, hourly workers without monthly pay, readable messages listing everything missing at once

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solutions/demo/closing-engine/template.xlsx
+++ b/solutions/demo/closing-engine/template.xlsx
@@ -2808,7 +2808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2825,6 +2825,7 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2898,6 +2899,11 @@
           <t>停车费</t>
         </is>
       </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>住民税(无特别征收填 none)</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1">
       <c r="A2" t="inlineStr">
@@ -2968,6 +2974,11 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>commute_parking</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>juminzei_method</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(closing): issues found by the first user test (an agent playing a first-time user)
- 确认・取消一张凭证时，别的行里填了还没确认的内容不再被清空
- 没有读取模板的单据：说明「还不能自动读取」，文件名可以点开原件对照着填
- 带着回答重新结账：先说清会写进工作文件夹里的公司资料.xlsx（原文件先备份）
- 结账期间：说明为什么默认是整个会计年度
- 回答表单的税区分占位：「按科目的默认」
- 三条「前提」类事项的建议改成外行能看懂的话（引擎 bef7ec5），通勤方式的表头与页面一致

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solutions/demo/closing-engine/template.xlsx
+++ b/solutions/demo/closing-engine/template.xlsx
@@ -2821,7 +2821,7 @@
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>通勤方式(car/transit)</t>
+          <t>通勤方式(transit/car/mixed)</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">

</xml_diff>